<commit_message>
Add new category and subcategories system
</commit_message>
<xml_diff>
--- a/client/src/templates/creatorFormTemplate.xlsx
+++ b/client/src/templates/creatorFormTemplate.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re9076a825f194d54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re588ab39376a4ddc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -558,7 +558,7 @@
       <x:c r="AC1"/>
       <x:c r="AD1"/>
     </x:row>
-    <x:row r="2" ht="49.5" customHeight="1">
+    <x:row r="2" ht="46" customHeight="1">
       <x:c r="A2" s="37" t="str">
         <x:v>Tự động</x:v>
       </x:c>
@@ -572,7 +572,7 @@
         <x:v>Mặc định MINI</x:v>
       </x:c>
       <x:c r="E2" s="42" t="str">
-        <x:v>Có thể nhập nhiều giá trị, ngăn cách bằng dấu phẩy · mặc định BEAUTY</x:v>
+        <x:v>Category tự do. Phân cấp bằng dấu &gt; · VD: Newborns &amp; Maternity &gt; Baby Product · nhiều nhánh: abc &gt; cde, fgh · để trống = OTHER</x:v>
       </x:c>
       <x:c r="F2" s="42" t="str">
         <x:v>Có thể nhập nhiều giá trị, ngăn cách bằng dấu phẩy · mặc định VIDEO</x:v>

</xml_diff>